<commit_message>
feat: restruturação de regras
</commit_message>
<xml_diff>
--- a/regras.xlsx
+++ b/regras.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="132">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -21,31 +21,31 @@
     <t>CAMINHO_BASE</t>
   </si>
   <si>
-    <t>2 L TRANSPORTES</t>
+    <t xml:space="preserve">2 L TRANSPORTES </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\2 L TRANSPORTES LTDA</t>
   </si>
   <si>
-    <t>ADELANE E FABIO</t>
+    <t xml:space="preserve">ADELANE E FABIO </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Adelane e Fabio Ltda</t>
   </si>
   <si>
-    <t>ADELSON ROSA</t>
+    <t xml:space="preserve">ADELSON ROSA </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Adelson Rosa Vaz</t>
   </si>
   <si>
-    <t>ADENIR ROSA VAZ</t>
+    <t xml:space="preserve">ADENIR VAZ </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Adenir Vaz Dos Santos Representacoes Ltda</t>
   </si>
   <si>
-    <t>ADILSON REZENDE</t>
+    <t xml:space="preserve">ADILSON REZENDE </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\PESSOA FÍSICA\FAZENDAS\Adilson Rezende Silva</t>
@@ -57,31 +57,31 @@
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\AE HOTELARIA</t>
   </si>
   <si>
-    <t>BESSA E GOMIDE</t>
+    <t xml:space="preserve">BESSA E GOMIDE </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Bessa e Gomide Ltda</t>
   </si>
   <si>
-    <t>BSMAG</t>
+    <t>BSMAG LTDA</t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Bsmag Ltda</t>
   </si>
   <si>
-    <t>CARVALHO REPRESENTAÇÕES</t>
+    <t xml:space="preserve">CARVALHO REPRESENTAÇÕES </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Carvalho Representacoes Ltda</t>
   </si>
   <si>
-    <t>CELERE CONSULTORIA</t>
+    <t xml:space="preserve">CELERE CONSULTORIA </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Celere Consultoria Empresarial Ltda</t>
   </si>
   <si>
-    <t>COMERCIAL FERNANDES</t>
+    <t xml:space="preserve">COMERCIAL FERNANDES </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Comercial Fernandes EIRELI</t>
@@ -93,28 +93,31 @@
     <t>P:\P\EMPRESAS\ATIVAS\IMUNE ISENTAS\COUNTRY CLUBE</t>
   </si>
   <si>
-    <t>HMC (CRESCI E PERDI)</t>
+    <t>H M C LTDA</t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\H M C Ltda</t>
   </si>
   <si>
-    <t>DEIVID DE OLIVEIRA</t>
+    <t>DEIVID CARTORIO</t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\PESSOA FÍSICA\DEMAIS\DEIVID DE OLIVEIRA RIBEIRO</t>
   </si>
   <si>
-    <t>DENISE CAMPOS</t>
+    <t xml:space="preserve">DENISE CAMPOS </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Denise Alcione Campos Silva Ltda</t>
   </si>
   <si>
-    <t>DROGARIA ALVES</t>
-  </si>
-  <si>
-    <t>ELAINE CRISTINA</t>
+    <t xml:space="preserve">DROGARIA ALVES </t>
+  </si>
+  <si>
+    <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Drogaria Alves Pharma Ltda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ELAINE CRISTINA </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\PESSOA FÍSICA\DOMESTICAS\ELAINE CRISTINA ROCHA GOULART</t>
@@ -123,43 +126,46 @@
     <t>EPM ALIMENTOS</t>
   </si>
   <si>
-    <t>EUDES MARÇAL</t>
+    <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Epm Alimentos Ltda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUDES MARCAL </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\PESSOA FÍSICA\FAZENDAS\EUDES MARCAL LELLIS</t>
   </si>
   <si>
-    <t>FABRICIO CARRIÃO</t>
+    <t xml:space="preserve">FABRICIO CARREAO </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\PESSOA FÍSICA\DOMESTICAS\FABRICIO CARREAO DOS SANTOS</t>
   </si>
   <si>
-    <t>FAZENDA TRÊS BARRAS</t>
+    <t xml:space="preserve">FAZENDA TRES BARRAS </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Fazenda Tres Barras Transportes e Prestação de Serviços Ltda</t>
   </si>
   <si>
-    <t>FFVA ENGENHARIA</t>
+    <t xml:space="preserve">FFVA ENGENHARIA </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\FFVA Engenharia Ltda</t>
   </si>
   <si>
-    <t>FLAVIO RIBEIRO</t>
+    <t xml:space="preserve">FLAVIO RIBEIRO </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Flavio Ribeiro de Menezes</t>
   </si>
   <si>
-    <t>GH FILIAL</t>
+    <t xml:space="preserve">GH AGROPECUARIA MATRIZ </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\LUCRO PRESUMIDO\G H AGROPECUARIA LTDA\MATRIZ\GH AGROPECUARIA LTDA</t>
   </si>
   <si>
-    <t>GH MATRIZ</t>
+    <t>GH AGROPECUARIA FILIAL</t>
   </si>
   <si>
     <t>GILMAR GOMES</t>
@@ -168,19 +174,19 @@
     <t>P:\P\EMPRESAS\ATIVAS\PESSOA FÍSICA\FAZENDAS\Gilmar Gomes dos Santos Junior</t>
   </si>
   <si>
-    <t>HENRIQUE LELLES</t>
+    <t xml:space="preserve">HENRIQUE LELLES </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\PESSOA FÍSICA\FAZENDAS\Henrique Lelles Bezerra</t>
   </si>
   <si>
-    <t>HOTEL GLOBO</t>
+    <t xml:space="preserve">HOTEL GLOBO </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Hotel Globo Ltda</t>
   </si>
   <si>
-    <t>HVM AGRO</t>
+    <t xml:space="preserve">HVM AGRO </t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\HVM AGRO REPRESENTAÇÕES LTDA</t>
@@ -204,13 +210,13 @@
     <t>P:\P\EMPRESAS\ATIVAS\PESSOA FÍSICA\FAZENDAS\Jose dos Reis Fazenda</t>
   </si>
   <si>
-    <t>KEYLA GEOVANNA</t>
+    <t>CARTORIO KEYLA</t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\IMUNE ISENTAS\SANTA CRUZ DE GOIAS CARTORIO 1º OFICIO-KEYLA</t>
   </si>
   <si>
-    <t>LEDA LENZA</t>
+    <t>LEDA</t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\PESSOA FÍSICA\DOMESTICAS\LEDA\2026</t>
@@ -246,7 +252,7 @@
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Maria Cecilia Da Silva Trindade Dias</t>
   </si>
   <si>
-    <t>MARIA TEREZA</t>
+    <t>MARIA TEREZA CARTORIO</t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\IMUNE ISENTAS\SANTA CRUZ DE GOIAS TABELIONATO DE NOTAS, DE PROTESTOS E DE TITULOS, TABELIA-MARIA TEREZA</t>
@@ -318,7 +324,7 @@
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Pousada Palmelo Ltda</t>
   </si>
   <si>
-    <t>PRONEXT T.I</t>
+    <t>PRONEXT</t>
   </si>
   <si>
     <t>P:\P\EMPRESAS\ATIVAS\SIMPLES NACIONAL\Pronext Tecnologia Ltda</t>
@@ -381,7 +387,7 @@
     <t>DP</t>
   </si>
   <si>
-    <t>RECORRENTE{ANO}\DEPARTAMENTO PESSOAL\RESUMO DA FOLHA</t>
+    <t>RECORRENTE\{ANO}\DEPARTAMENTO PESSOAL\RESUMO DA FOLHA</t>
   </si>
   <si>
     <t>INSS</t>
@@ -390,9 +396,6 @@
     <t>FOLHA</t>
   </si>
   <si>
-    <t>RECORRENTE\{ANO}\DEPARTAMENTO PESSOAL\RESUMO DA FOLHA</t>
-  </si>
-  <si>
     <t>PALAVRA_CHAVE</t>
   </si>
   <si>
@@ -403,6 +406,9 @@
   </si>
   <si>
     <t>RESUMO DA FOLHA</t>
+  </si>
+  <si>
+    <t>RECIBO DE PAGAMENTO</t>
   </si>
 </sst>
 </file>
@@ -455,7 +461,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -467,6 +473,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
@@ -823,7 +832,7 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="34.43"/>
+    <col customWidth="1" min="1" max="1" width="38.14"/>
     <col customWidth="1" min="2" max="2" width="155.29"/>
     <col customWidth="1" min="3" max="26" width="8.71"/>
   </cols>
@@ -864,7 +873,7 @@
       <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="5" t="s">
         <v>3</v>
       </c>
     </row>
@@ -872,7 +881,7 @@
       <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
     </row>
@@ -880,7 +889,7 @@
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="5" t="s">
         <v>7</v>
       </c>
     </row>
@@ -888,7 +897,7 @@
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>9</v>
       </c>
     </row>
@@ -896,15 +905,15 @@
       <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>13</v>
       </c>
     </row>
@@ -912,7 +921,7 @@
       <c r="A8" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B8" s="5" t="s">
         <v>15</v>
       </c>
     </row>
@@ -920,7 +929,7 @@
       <c r="A9" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>17</v>
       </c>
     </row>
@@ -928,7 +937,7 @@
       <c r="A10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B10" s="5" t="s">
         <v>19</v>
       </c>
     </row>
@@ -936,7 +945,7 @@
       <c r="A11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>21</v>
       </c>
     </row>
@@ -944,15 +953,15 @@
       <c r="A12" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B12" s="5" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" ht="22.5" customHeight="1">
-      <c r="A13" s="4" t="s">
+      <c r="A13" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>25</v>
       </c>
     </row>
@@ -960,7 +969,7 @@
       <c r="A14" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B14" s="5" t="s">
         <v>27</v>
       </c>
     </row>
@@ -968,7 +977,7 @@
       <c r="A15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>29</v>
       </c>
     </row>
@@ -976,7 +985,7 @@
       <c r="A16" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="5" t="s">
         <v>31</v>
       </c>
     </row>
@@ -985,356 +994,356 @@
         <v>32</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="B18" s="4" t="s">
         <v>34</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>31</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="A22" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>43</v>
+        <v>44</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>47</v>
+        <v>50</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>58</v>
+      <c r="A31" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>60</v>
+      <c r="A32" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>62</v>
+      <c r="A33" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="A34" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="A35" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>68</v>
+      <c r="A36" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>70</v>
+      <c r="A37" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>72</v>
+      <c r="A38" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>74</v>
+      <c r="A39" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>76</v>
+      <c r="A40" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="A41" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>80</v>
+      <c r="A42" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>82</v>
+      <c r="A43" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>84</v>
+      <c r="A44" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>86</v>
+      <c r="A45" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>88</v>
+      <c r="A46" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>90</v>
+      <c r="A47" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>92</v>
+      <c r="A48" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>94</v>
+      <c r="A49" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>96</v>
+      <c r="A50" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="B50" s="5" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>98</v>
+      <c r="A51" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B51" s="5" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>100</v>
+      <c r="A52" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="B52" s="5" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="A53" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
+      </c>
+      <c r="B53" s="5" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>104</v>
+      <c r="A54" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B54" s="5" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>106</v>
+      <c r="A55" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="B55" s="5" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>108</v>
+      <c r="A56" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="B56" s="5" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>110</v>
+      <c r="A57" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B58" s="4" t="s">
-        <v>112</v>
+      <c r="A58" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="4" t="s">
-        <v>113</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>114</v>
+      <c r="A59" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>116</v>
+      <c r="A60" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B60" s="5" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="5"/>
-      <c r="B61" s="6"/>
+      <c r="A61" s="6"/>
+      <c r="B61" s="7"/>
     </row>
     <row r="62" ht="15.75" customHeight="1"/>
     <row r="63" ht="15.75" customHeight="1"/>
@@ -2274,7 +2283,6 @@
     <row r="997" ht="15.75" customHeight="1"/>
     <row r="998" ht="15.75" customHeight="1"/>
     <row r="999" ht="15.75" customHeight="1"/>
-    <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <printOptions/>
   <pageMargins bottom="1.0" footer="0.0" header="0.0" left="0.75" right="0.75" top="1.0"/>
@@ -2301,53 +2309,53 @@
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="B1" s="7" t="s">
-        <v>118</v>
-      </c>
-      <c r="C1" s="7" t="s">
+      <c r="A1" s="8" t="s">
         <v>119</v>
       </c>
+      <c r="B1" s="8" t="s">
+        <v>120</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>121</v>
+      </c>
     </row>
     <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" s="9" t="s">
+      <c r="A2" s="9" t="s">
         <v>122</v>
       </c>
+      <c r="B2" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>124</v>
+      </c>
     </row>
     <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="8" t="s">
+      <c r="A3" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>122</v>
+      <c r="C3" s="10" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="9" t="s">
+        <v>126</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>125</v>
-      </c>
     </row>
     <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -3348,70 +3356,74 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="23.14"/>
+    <col customWidth="1" min="1" max="1" width="25.86"/>
     <col customWidth="1" min="2" max="2" width="24.57"/>
     <col customWidth="1" min="3" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="22.5" customHeight="1">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="9" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" ht="22.5" customHeight="1">
-      <c r="A2" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="3" ht="22.5" customHeight="1">
-      <c r="A3" s="8" t="s">
-        <v>127</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="4" ht="22.5" customHeight="1">
-      <c r="A4" s="8" t="s">
-        <v>123</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="5" ht="22.5" customHeight="1">
-      <c r="A5" s="8" t="s">
-        <v>128</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="6" ht="22.5" customHeight="1">
-      <c r="A6" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>124</v>
+      <c r="B6" s="9" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="7" ht="22.5" customHeight="1">
-      <c r="A7" s="8" t="s">
-        <v>129</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>124</v>
+      <c r="A7" s="9" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="8" ht="22.5" customHeight="1">
-      <c r="A8" s="10"/>
-      <c r="B8" s="11"/>
+      <c r="A8" s="11" t="s">
+        <v>131</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>
     <row r="22" ht="15.75" customHeight="1"/>

</xml_diff>